<commit_message>
Add AR measurement export and placement support
</commit_message>
<xml_diff>
--- a/Construction_Engineering_Project_Log.xlsx
+++ b/Construction_Engineering_Project_Log.xlsx
@@ -669,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M216"/>
+  <dimension ref="A1:M217"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="13" customWidth="1" style="21" min="1" max="1"/>
@@ -1099,111 +1099,241 @@
       <c r="M13" s="5" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="n"/>
-      <c r="B14" s="19" t="n"/>
-      <c r="C14" s="19" t="n"/>
+      <c r="A14" s="17" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B14" s="19" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="C14" s="19" t="n">
+        <v>0.4166666666666667</v>
+      </c>
       <c r="D14" s="14">
         <f>IF(OR(B14="",C14=""),"",MOD(C14-B14,1)*24)</f>
         <v/>
       </c>
-      <c r="E14" s="20" t="n"/>
-      <c r="F14" s="20" t="n"/>
-      <c r="G14" s="20" t="n"/>
-      <c r="H14" s="20" t="n"/>
+      <c r="E14" s="20" t="inlineStr">
+        <is>
+          <t>Measurement</t>
+        </is>
+      </c>
+      <c r="F14" s="20" t="inlineStr">
+        <is>
+          <t>Reworked the AR measurement capture model to use a center reticle and explicit point capture flow instead of direct tap placement.</t>
+        </is>
+      </c>
+      <c r="G14" s="20" t="inlineStr">
+        <is>
+          <t>construction-ar-platform/ios/ConstructionARPlatform/MeasurementARView.swift; construction-ar-platform/src/features/measurement/NativeMeasurementARView.tsx</t>
+        </is>
+      </c>
+      <c r="H14" s="20" t="inlineStr">
+        <is>
+          <t>eeb95b31</t>
+        </is>
+      </c>
       <c r="I14" s="20" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J14" s="20" t="n"/>
+      <c r="J14" s="20" t="inlineStr">
+        <is>
+          <t>Added reticle state, tracking feedback, and Point A / Point B capture handling for defensible targeting.</t>
+        </is>
+      </c>
       <c r="K14" s="5" t="n"/>
       <c r="L14" s="5" t="n"/>
       <c r="M14" s="5" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="n"/>
-      <c r="B15" s="19" t="n"/>
-      <c r="C15" s="19" t="n"/>
+      <c r="A15" s="17" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B15" s="19" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="C15" s="19" t="n">
+        <v>0.4583333333333333</v>
+      </c>
       <c r="D15" s="14">
         <f>IF(OR(B15="",C15=""),"",MOD(C15-B15,1)*24)</f>
         <v/>
       </c>
-      <c r="E15" s="20" t="n"/>
-      <c r="F15" s="20" t="n"/>
-      <c r="G15" s="20" t="n"/>
-      <c r="H15" s="20" t="n"/>
+      <c r="E15" s="20" t="inlineStr">
+        <is>
+          <t>Measurement</t>
+        </is>
+      </c>
+      <c r="F15" s="20" t="inlineStr">
+        <is>
+          <t>Wired the revised measurement workspace into the app with project and room selection, live status messaging, and the AR measurement screen flow.</t>
+        </is>
+      </c>
+      <c r="G15" s="20" t="inlineStr">
+        <is>
+          <t>construction-ar-platform/src/features/measurement/MeasurementScreen.tsx; construction-ar-platform/src/app/AppShell.tsx</t>
+        </is>
+      </c>
+      <c r="H15" s="20" t="inlineStr">
+        <is>
+          <t>eeb95b31</t>
+        </is>
+      </c>
       <c r="I15" s="20" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J15" s="20" t="n"/>
+      <c r="J15" s="20" t="inlineStr">
+        <is>
+          <t>Connected the new measurement screen to the mobile app shell and room-scoped measuring workflow.</t>
+        </is>
+      </c>
       <c r="K15" s="5" t="n"/>
       <c r="L15" s="5" t="n"/>
       <c r="M15" s="5" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="n"/>
-      <c r="B16" s="19" t="n"/>
-      <c r="C16" s="19" t="n"/>
+      <c r="A16" s="17" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B16" s="19" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="C16" s="19" t="n">
+        <v>0.4166666666666667</v>
+      </c>
       <c r="D16" s="14">
         <f>IF(OR(B16="",C16=""),"",MOD(C16-B16,1)*24)</f>
         <v/>
       </c>
-      <c r="E16" s="20" t="n"/>
-      <c r="F16" s="20" t="n"/>
-      <c r="G16" s="20" t="n"/>
-      <c r="H16" s="20" t="n"/>
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t>Measurement</t>
+        </is>
+      </c>
+      <c r="F16" s="20" t="inlineStr">
+        <is>
+          <t>Built the multi-capture measurement flow so repeated passes can be collected, reviewed, and resolved into a single result.</t>
+        </is>
+      </c>
+      <c r="G16" s="20" t="inlineStr">
+        <is>
+          <t>construction-ar-platform/src/features/measurement/MeasurementScreen.tsx; construction-ar-platform/src/domain/measurements.ts</t>
+        </is>
+      </c>
+      <c r="H16" s="20" t="inlineStr">
+        <is>
+          <t>eeb95b31</t>
+        </is>
+      </c>
       <c r="I16" s="20" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J16" s="20" t="n"/>
+      <c r="J16" s="20" t="inlineStr">
+        <is>
+          <t>Implemented pass accumulation, add-another-pass handling, finish flow, and outlier-aware resolution for repeated captures.</t>
+        </is>
+      </c>
       <c r="K16" s="5" t="n"/>
       <c r="L16" s="5" t="n"/>
       <c r="M16" s="5" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="n"/>
-      <c r="B17" s="19" t="n"/>
-      <c r="C17" s="19" t="n"/>
+      <c r="A17" s="17" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B17" s="19" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="C17" s="19" t="n">
+        <v>0.4583333333333333</v>
+      </c>
       <c r="D17" s="14">
         <f>IF(OR(B17="",C17=""),"",MOD(C17-B17,1)*24)</f>
         <v/>
       </c>
-      <c r="E17" s="20" t="n"/>
-      <c r="F17" s="20" t="n"/>
-      <c r="G17" s="20" t="n"/>
-      <c r="H17" s="20" t="n"/>
+      <c r="E17" s="20" t="inlineStr">
+        <is>
+          <t>Measurement</t>
+        </is>
+      </c>
+      <c r="F17" s="20" t="inlineStr">
+        <is>
+          <t>Added the room-grouped measurement log with detail views and destructive actions for single entries, room groups, and the full log.</t>
+        </is>
+      </c>
+      <c r="G17" s="20" t="inlineStr">
+        <is>
+          <t>construction-ar-platform/src/features/measurement/MeasurementScreen.tsx; construction-ar-platform/src/domain/measurementLog.ts</t>
+        </is>
+      </c>
+      <c r="H17" s="20" t="inlineStr">
+        <is>
+          <t>eeb95b31</t>
+        </is>
+      </c>
       <c r="I17" s="20" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J17" s="20" t="n"/>
+      <c r="J17" s="20" t="inlineStr">
+        <is>
+          <t>Supports single-entry delete, Clear Room, Clear All, and room-based grouping tied to existing project rooms.</t>
+        </is>
+      </c>
       <c r="K17" s="5" t="n"/>
       <c r="L17" s="5" t="n"/>
       <c r="M17" s="5" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="n"/>
-      <c r="B18" s="19" t="n"/>
-      <c r="C18" s="19" t="n"/>
+      <c r="A18" s="17" t="n">
+        <v>46250</v>
+      </c>
+      <c r="B18" s="19" t="n">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="C18" s="19" t="n">
+        <v>0.5</v>
+      </c>
       <c r="D18" s="14">
         <f>IF(OR(B18="",C18=""),"",MOD(C18-B18,1)*24)</f>
         <v/>
       </c>
-      <c r="E18" s="20" t="n"/>
-      <c r="F18" s="20" t="n"/>
-      <c r="G18" s="20" t="n"/>
-      <c r="H18" s="20" t="n"/>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>Measurement</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>Standardized measurement output to decimal inches and added supporting log, persistence, and measurement tests around the new workflow.</t>
+        </is>
+      </c>
+      <c r="G18" s="20" t="inlineStr">
+        <is>
+          <t>construction-ar-platform/src/domain/measurementUnits.ts; construction-ar-platform/src/domain/measurementLog.test.ts; construction-ar-platform/src/domain/measurements.test.ts; construction-ar-platform/src/storage/projectDocument.ts</t>
+        </is>
+      </c>
+      <c r="H18" s="20" t="inlineStr">
+        <is>
+          <t>eeb95b31</t>
+        </is>
+      </c>
       <c r="I18" s="20" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J18" s="20" t="n"/>
+      <c r="J18" s="20" t="inlineStr">
+        <is>
+          <t>Locked the UI to inches-only display labels and covered the new measurement/log model with regression tests; calibration still ongoing.</t>
+        </is>
+      </c>
       <c r="K18" s="5" t="n"/>
       <c r="L18" s="5" t="n"/>
       <c r="M18" s="5" t="n"/>
@@ -5678,7 +5808,18 @@
         </is>
       </c>
     </row>
-    <row r="217" ht="15.75" customHeight="1" s="21"/>
+    <row r="217" ht="15.75" customHeight="1" s="21">
+      <c r="A217" s="17" t="n"/>
+      <c r="B217" s="19" t="n"/>
+      <c r="C217" s="19" t="n"/>
+      <c r="D217" s="14" t="n"/>
+      <c r="E217" s="20" t="n"/>
+      <c r="F217" s="20" t="n"/>
+      <c r="G217" s="20" t="n"/>
+      <c r="H217" s="20" t="n"/>
+      <c r="I217" s="20" t="n"/>
+      <c r="J217" s="20" t="n"/>
+    </row>
     <row r="218" ht="15.75" customHeight="1" s="21"/>
     <row r="219" ht="15.75" customHeight="1" s="21"/>
     <row r="220" ht="15.75" customHeight="1" s="21"/>

</xml_diff>